<commit_message>
Fix model outputs with correct data format, update figures
</commit_message>
<xml_diff>
--- a/Analysis/clean data/Formatted for viewing_Survey 1 & 2_scored_near complete_16.6.26.xlsx
+++ b/Analysis/clean data/Formatted for viewing_Survey 1 & 2_scored_near complete_16.6.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ranidavis/Desktop/Bats &amp; agriculture/Beneficial Bats - collaborative paper/IBRC paper analysis/IBRC beneficial bats survey response analysis/Analysis/clean data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB70CAF-74FB-9E45-A107-0283CE47A29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09048272-3F30-154E-9513-10AF5ED772AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35560" yWindow="-2100" windowWidth="33120" windowHeight="19380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2446,9 +2446,6 @@
     <t>Tried, not tested - water sources have been created, but knowledge of its benefits to bats in this system is anecdotal or theoretical</t>
   </si>
   <si>
-    <t>AS</t>
-  </si>
-  <si>
     <t>Vineyards, Chile</t>
   </si>
   <si>
@@ -3163,6 +3160,9 @@
   </si>
   <si>
     <t>R44</t>
+  </si>
+  <si>
+    <t>AMS</t>
   </si>
 </sst>
 </file>
@@ -12862,7 +12862,7 @@
         <v>38</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>790</v>
+        <v>1027</v>
       </c>
       <c r="C4" s="46" t="s">
         <v>85</v>
@@ -12892,16 +12892,16 @@
         <v>88</v>
       </c>
       <c r="L4" s="1" t="s">
+        <v>1027</v>
+      </c>
+      <c r="M4" s="45" t="s">
         <v>790</v>
-      </c>
-      <c r="M4" s="45" t="s">
-        <v>791</v>
       </c>
       <c r="N4" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O4" s="45" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="P4" s="45" t="s">
         <v>787</v>
@@ -12910,13 +12910,13 @@
         <v>788</v>
       </c>
       <c r="S4" s="45" t="s">
+        <v>792</v>
+      </c>
+      <c r="T4" s="45" t="s">
         <v>793</v>
       </c>
-      <c r="T4" s="45" t="s">
+      <c r="V4" s="45" t="s">
         <v>794</v>
-      </c>
-      <c r="V4" s="45" t="s">
-        <v>795</v>
       </c>
       <c r="X4" s="45" t="s">
         <v>783</v>
@@ -12978,43 +12978,43 @@
         <v>714</v>
       </c>
       <c r="M5" s="45" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="N5" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O5" s="45" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="P5" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q5" s="45" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="R5" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S5" s="45" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="T5" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U5" s="45" t="s">
+        <v>799</v>
+      </c>
+      <c r="V5" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W5" s="45" t="s">
         <v>800</v>
       </c>
-      <c r="V5" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W5" s="45" t="s">
+      <c r="X5" s="45" t="s">
         <v>801</v>
       </c>
-      <c r="X5" s="45" t="s">
+      <c r="Y5" s="45" t="s">
         <v>802</v>
-      </c>
-      <c r="Y5" s="45" t="s">
-        <v>803</v>
       </c>
       <c r="Z5" s="47">
         <v>1</v>
@@ -13073,31 +13073,31 @@
         <v>713</v>
       </c>
       <c r="M6" s="45" t="s">
+        <v>803</v>
+      </c>
+      <c r="N6" s="45" t="s">
         <v>804</v>
-      </c>
-      <c r="N6" s="45" t="s">
-        <v>805</v>
       </c>
       <c r="P6" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q6" s="45" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="R6" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S6" s="45" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="T6" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U6" s="45" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="V6" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X6" s="45" t="s">
         <v>783</v>
@@ -13159,40 +13159,40 @@
         <v>715</v>
       </c>
       <c r="M7" s="45" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="N7" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O7" s="45" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="P7" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q7" s="45" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="R7" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S7" s="45" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="T7" s="45" t="s">
+        <v>811</v>
+      </c>
+      <c r="U7" s="45" t="s">
         <v>812</v>
       </c>
-      <c r="U7" s="45" t="s">
-        <v>813</v>
-      </c>
       <c r="V7" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X7" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y7" s="45" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="Z7" s="47">
         <v>1</v>
@@ -13224,7 +13224,7 @@
         <v>144</v>
       </c>
       <c r="D8" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E8" s="45" t="s">
         <v>158</v>
@@ -13251,13 +13251,13 @@
         <v>716</v>
       </c>
       <c r="M8" s="45" t="s">
+        <v>815</v>
+      </c>
+      <c r="N8" s="45" t="s">
         <v>816</v>
       </c>
-      <c r="N8" s="45" t="s">
+      <c r="O8" s="45" t="s">
         <v>817</v>
-      </c>
-      <c r="O8" s="45" t="s">
-        <v>818</v>
       </c>
       <c r="P8" s="45" t="s">
         <v>775</v>
@@ -13269,13 +13269,13 @@
         <v>779</v>
       </c>
       <c r="U8" s="45" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="V8" s="45" t="s">
         <v>781</v>
       </c>
       <c r="W8" s="45" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="X8" s="45" t="s">
         <v>783</v>
@@ -13337,7 +13337,7 @@
         <v>716</v>
       </c>
       <c r="M9" s="45" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="N9" s="45" t="s">
         <v>773</v>
@@ -13352,10 +13352,10 @@
         <v>779</v>
       </c>
       <c r="U9" s="45" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="V9" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X9" s="45" t="s">
         <v>783</v>
@@ -13390,7 +13390,7 @@
         <v>172</v>
       </c>
       <c r="D10" s="46" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="E10" s="45" t="s">
         <v>225</v>
@@ -13417,25 +13417,25 @@
         <v>717</v>
       </c>
       <c r="M10" s="45" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="N10" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P10" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q10" s="45" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="R10" s="45" t="s">
         <v>788</v>
       </c>
       <c r="T10" s="45" t="s">
+        <v>793</v>
+      </c>
+      <c r="V10" s="45" t="s">
         <v>794</v>
-      </c>
-      <c r="V10" s="45" t="s">
-        <v>795</v>
       </c>
       <c r="X10" s="45" t="s">
         <v>783</v>
@@ -13497,37 +13497,37 @@
         <v>717</v>
       </c>
       <c r="M11" s="45" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="N11" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O11" s="45" t="s">
+        <v>826</v>
+      </c>
+      <c r="P11" s="45" t="s">
         <v>827</v>
       </c>
-      <c r="P11" s="45" t="s">
+      <c r="Q11" s="45" t="s">
         <v>828</v>
       </c>
-      <c r="Q11" s="45" t="s">
+      <c r="R11" s="45" t="s">
         <v>829</v>
       </c>
-      <c r="R11" s="45" t="s">
+      <c r="S11" s="45" t="s">
         <v>830</v>
       </c>
-      <c r="S11" s="45" t="s">
+      <c r="T11" s="45" t="s">
+        <v>811</v>
+      </c>
+      <c r="U11" s="45" t="s">
         <v>831</v>
-      </c>
-      <c r="T11" s="45" t="s">
-        <v>812</v>
-      </c>
-      <c r="U11" s="45" t="s">
-        <v>832</v>
       </c>
       <c r="V11" s="45" t="s">
         <v>781</v>
       </c>
       <c r="W11" s="45" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="X11" s="45" t="s">
         <v>783</v>
@@ -13562,10 +13562,10 @@
         <v>172</v>
       </c>
       <c r="D12" s="46" t="s">
+        <v>833</v>
+      </c>
+      <c r="E12" s="45" t="s">
         <v>834</v>
-      </c>
-      <c r="E12" s="45" t="s">
-        <v>835</v>
       </c>
       <c r="F12" s="45" t="s">
         <v>174</v>
@@ -13592,13 +13592,13 @@
         <v>70</v>
       </c>
       <c r="N12" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P12" s="45" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="Q12" s="45" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="R12" s="45" t="s">
         <v>788</v>
@@ -13607,19 +13607,19 @@
         <v>779</v>
       </c>
       <c r="U12" s="45" t="s">
+        <v>836</v>
+      </c>
+      <c r="V12" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W12" s="45" t="s">
         <v>837</v>
-      </c>
-      <c r="V12" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W12" s="45" t="s">
-        <v>838</v>
       </c>
       <c r="X12" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y12" s="45" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="Z12" s="47">
         <v>0</v>
@@ -13651,10 +13651,10 @@
         <v>172</v>
       </c>
       <c r="D13" s="46" t="s">
+        <v>839</v>
+      </c>
+      <c r="E13" s="45" t="s">
         <v>840</v>
-      </c>
-      <c r="E13" s="45" t="s">
-        <v>841</v>
       </c>
       <c r="F13" s="45" t="s">
         <v>174</v>
@@ -13684,13 +13684,13 @@
         <v>773</v>
       </c>
       <c r="O13" s="45" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="P13" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q13" s="45" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="R13" s="45" t="s">
         <v>788</v>
@@ -13699,19 +13699,19 @@
         <v>779</v>
       </c>
       <c r="U13" s="45" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="V13" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W13" s="45" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="X13" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y13" s="45" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="Z13" s="47">
         <v>1</v>
@@ -13743,10 +13743,10 @@
         <v>172</v>
       </c>
       <c r="D14" s="46" t="s">
+        <v>845</v>
+      </c>
+      <c r="E14" s="45" t="s">
         <v>846</v>
-      </c>
-      <c r="E14" s="45" t="s">
-        <v>847</v>
       </c>
       <c r="F14" s="45" t="s">
         <v>174</v>
@@ -13773,13 +13773,13 @@
         <v>214</v>
       </c>
       <c r="N14" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P14" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q14" s="45" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="R14" s="45" t="s">
         <v>788</v>
@@ -13788,19 +13788,19 @@
         <v>779</v>
       </c>
       <c r="U14" s="45" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="V14" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W14" s="45" t="s">
+        <v>848</v>
+      </c>
+      <c r="X14" s="45" t="s">
         <v>849</v>
       </c>
-      <c r="X14" s="45" t="s">
+      <c r="Y14" s="45" t="s">
         <v>850</v>
-      </c>
-      <c r="Y14" s="45" t="s">
-        <v>851</v>
       </c>
       <c r="Z14" s="47">
         <v>0</v>
@@ -13832,10 +13832,10 @@
         <v>172</v>
       </c>
       <c r="D15" s="46" t="s">
+        <v>845</v>
+      </c>
+      <c r="E15" s="45" t="s">
         <v>846</v>
-      </c>
-      <c r="E15" s="45" t="s">
-        <v>847</v>
       </c>
       <c r="F15" s="45" t="s">
         <v>174</v>
@@ -13862,10 +13862,10 @@
         <v>214</v>
       </c>
       <c r="N15" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="O15" s="45" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="P15" s="45" t="s">
         <v>775</v>
@@ -13877,10 +13877,10 @@
         <v>779</v>
       </c>
       <c r="V15" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X15" s="45" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="Z15" s="47">
         <v>0</v>
@@ -13912,7 +13912,7 @@
         <v>172</v>
       </c>
       <c r="D16" s="46" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="E16" s="45" t="s">
         <v>173</v>
@@ -13939,13 +13939,13 @@
         <v>717</v>
       </c>
       <c r="M16" s="45" t="s">
+        <v>853</v>
+      </c>
+      <c r="N16" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O16" s="45" t="s">
         <v>854</v>
-      </c>
-      <c r="N16" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O16" s="45" t="s">
-        <v>855</v>
       </c>
       <c r="P16" s="45" t="s">
         <v>787</v>
@@ -13957,19 +13957,19 @@
         <v>779</v>
       </c>
       <c r="U16" s="45" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="V16" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W16" s="45" t="s">
+        <v>855</v>
+      </c>
+      <c r="X16" s="45" t="s">
+        <v>849</v>
+      </c>
+      <c r="Y16" s="45" t="s">
         <v>856</v>
-      </c>
-      <c r="X16" s="45" t="s">
-        <v>850</v>
-      </c>
-      <c r="Y16" s="45" t="s">
-        <v>857</v>
       </c>
       <c r="Z16" s="47">
         <v>0</v>
@@ -14001,7 +14001,7 @@
         <v>172</v>
       </c>
       <c r="D17" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E17" s="45" t="s">
         <v>173</v>
@@ -14031,10 +14031,10 @@
         <v>186</v>
       </c>
       <c r="N17" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="O17" s="45" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="P17" s="45" t="s">
         <v>787</v>
@@ -14046,19 +14046,19 @@
         <v>779</v>
       </c>
       <c r="U17" s="45" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="V17" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W17" s="45" t="s">
+        <v>855</v>
+      </c>
+      <c r="X17" s="45" t="s">
+        <v>849</v>
+      </c>
+      <c r="Y17" s="45" t="s">
         <v>856</v>
-      </c>
-      <c r="X17" s="45" t="s">
-        <v>850</v>
-      </c>
-      <c r="Y17" s="45" t="s">
-        <v>857</v>
       </c>
       <c r="Z17" s="47">
         <v>0</v>
@@ -14090,10 +14090,10 @@
         <v>172</v>
       </c>
       <c r="D18" s="46" t="s">
+        <v>858</v>
+      </c>
+      <c r="E18" s="45" t="s">
         <v>859</v>
-      </c>
-      <c r="E18" s="45" t="s">
-        <v>860</v>
       </c>
       <c r="F18" s="45" t="s">
         <v>174</v>
@@ -14120,16 +14120,16 @@
         <v>191</v>
       </c>
       <c r="N18" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="O18" s="45" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="P18" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q18" s="45" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="R18" s="45" t="s">
         <v>788</v>
@@ -14138,19 +14138,19 @@
         <v>779</v>
       </c>
       <c r="U18" s="45" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="V18" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W18" s="45" t="s">
+        <v>855</v>
+      </c>
+      <c r="X18" s="45" t="s">
+        <v>849</v>
+      </c>
+      <c r="Y18" s="45" t="s">
         <v>856</v>
-      </c>
-      <c r="X18" s="45" t="s">
-        <v>850</v>
-      </c>
-      <c r="Y18" s="45" t="s">
-        <v>857</v>
       </c>
       <c r="Z18" s="47">
         <v>0</v>
@@ -14182,7 +14182,7 @@
         <v>172</v>
       </c>
       <c r="D19" s="46" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E19" s="45" t="s">
         <v>173</v>
@@ -14212,40 +14212,40 @@
         <v>191</v>
       </c>
       <c r="N19" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="O19" s="45" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="P19" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q19" s="45" t="s">
+        <v>862</v>
+      </c>
+      <c r="R19" s="45" t="s">
+        <v>829</v>
+      </c>
+      <c r="S19" s="45" t="s">
         <v>863</v>
-      </c>
-      <c r="R19" s="45" t="s">
-        <v>830</v>
-      </c>
-      <c r="S19" s="45" t="s">
-        <v>864</v>
       </c>
       <c r="T19" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U19" s="45" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="V19" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W19" s="45" t="s">
+        <v>855</v>
+      </c>
+      <c r="X19" s="45" t="s">
+        <v>849</v>
+      </c>
+      <c r="Y19" s="45" t="s">
         <v>856</v>
-      </c>
-      <c r="X19" s="45" t="s">
-        <v>850</v>
-      </c>
-      <c r="Y19" s="45" t="s">
-        <v>857</v>
       </c>
       <c r="Z19" s="47">
         <v>0</v>
@@ -14277,10 +14277,10 @@
         <v>172</v>
       </c>
       <c r="D20" s="46" t="s">
+        <v>845</v>
+      </c>
+      <c r="E20" s="45" t="s">
         <v>846</v>
-      </c>
-      <c r="E20" s="45" t="s">
-        <v>847</v>
       </c>
       <c r="F20" s="45" t="s">
         <v>174</v>
@@ -14307,25 +14307,25 @@
         <v>214</v>
       </c>
       <c r="N20" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P20" s="45" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="Q20" s="45" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="R20" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S20" s="45" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="T20" s="45" t="s">
         <v>779</v>
       </c>
       <c r="V20" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="Z20" s="47">
         <v>0</v>
@@ -14354,7 +14354,7 @@
         <v>289</v>
       </c>
       <c r="D21" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E21" s="45" t="s">
         <v>304</v>
@@ -14381,34 +14381,34 @@
         <v>718</v>
       </c>
       <c r="M21" s="45" t="s">
+        <v>866</v>
+      </c>
+      <c r="N21" s="45" t="s">
+        <v>816</v>
+      </c>
+      <c r="O21" s="45" t="s">
         <v>867</v>
       </c>
-      <c r="N21" s="45" t="s">
-        <v>817</v>
-      </c>
-      <c r="O21" s="45" t="s">
+      <c r="P21" s="45" t="s">
+        <v>827</v>
+      </c>
+      <c r="Q21" s="45" t="s">
         <v>868</v>
       </c>
-      <c r="P21" s="45" t="s">
-        <v>828</v>
-      </c>
-      <c r="Q21" s="45" t="s">
+      <c r="R21" s="45" t="s">
+        <v>829</v>
+      </c>
+      <c r="S21" s="45" t="s">
         <v>869</v>
       </c>
-      <c r="R21" s="45" t="s">
-        <v>830</v>
-      </c>
-      <c r="S21" s="45" t="s">
-        <v>870</v>
-      </c>
       <c r="T21" s="45" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="V21" s="45" t="s">
         <v>781</v>
       </c>
       <c r="X21" s="45" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="Z21" s="47">
         <v>3</v>
@@ -14467,31 +14467,31 @@
         <v>718</v>
       </c>
       <c r="M22" s="45" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="N22" s="45" t="s">
         <v>785</v>
       </c>
       <c r="O22" s="45" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="P22" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q22" s="45" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R22" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S22" s="45" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="T22" s="45" t="s">
         <v>779</v>
       </c>
       <c r="V22" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X22" s="45" t="s">
         <v>783</v>
@@ -14553,10 +14553,10 @@
         <v>719</v>
       </c>
       <c r="M23" s="45" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="N23" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P23" s="45" t="s">
         <v>787</v>
@@ -14568,7 +14568,7 @@
         <v>779</v>
       </c>
       <c r="V23" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X23" s="45" t="s">
         <v>783</v>
@@ -14630,28 +14630,28 @@
         <v>720</v>
       </c>
       <c r="M24" s="45" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="N24" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P24" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q24" s="45" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="R24" s="45" t="s">
         <v>777</v>
       </c>
       <c r="T24" s="45" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="U24" s="45" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="V24" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X24" s="45" t="s">
         <v>783</v>
@@ -14713,25 +14713,25 @@
         <v>721</v>
       </c>
       <c r="N25" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P25" s="45" t="s">
+        <v>879</v>
+      </c>
+      <c r="Q25" s="45" t="s">
         <v>880</v>
-      </c>
-      <c r="Q25" s="45" t="s">
-        <v>881</v>
       </c>
       <c r="R25" s="45" t="s">
         <v>788</v>
       </c>
       <c r="T25" s="45" t="s">
+        <v>881</v>
+      </c>
+      <c r="U25" s="45" t="s">
         <v>882</v>
       </c>
-      <c r="U25" s="45" t="s">
-        <v>883</v>
-      </c>
       <c r="V25" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X25" s="45" t="s">
         <v>783</v>
@@ -14766,7 +14766,7 @@
         <v>346</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="E26" s="45" t="s">
         <v>347</v>
@@ -14793,13 +14793,13 @@
         <v>722</v>
       </c>
       <c r="M26" s="45" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="N26" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O26" s="45" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="P26" s="45" t="s">
         <v>787</v>
@@ -14808,16 +14808,16 @@
         <v>777</v>
       </c>
       <c r="S26" s="45" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="T26" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U26" s="45" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="V26" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X26" s="45" t="s">
         <v>783</v>
@@ -14879,31 +14879,31 @@
         <v>723</v>
       </c>
       <c r="M27" s="45" t="s">
+        <v>888</v>
+      </c>
+      <c r="N27" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O27" s="45" t="s">
         <v>889</v>
-      </c>
-      <c r="N27" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O27" s="45" t="s">
-        <v>890</v>
       </c>
       <c r="P27" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q27" s="45" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="R27" s="45" t="s">
         <v>788</v>
       </c>
       <c r="T27" s="45" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="U27" s="45" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="V27" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X27" s="45" t="s">
         <v>783</v>
@@ -14938,7 +14938,7 @@
         <v>389</v>
       </c>
       <c r="D28" s="46" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E28" s="45" t="s">
         <v>390</v>
@@ -14965,43 +14965,43 @@
         <v>724</v>
       </c>
       <c r="M28" s="45" t="s">
+        <v>892</v>
+      </c>
+      <c r="N28" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O28" s="45" t="s">
         <v>893</v>
-      </c>
-      <c r="N28" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O28" s="45" t="s">
-        <v>894</v>
       </c>
       <c r="P28" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q28" s="45" t="s">
+        <v>894</v>
+      </c>
+      <c r="R28" s="45" t="s">
         <v>895</v>
       </c>
-      <c r="R28" s="45" t="s">
+      <c r="S28" s="45" t="s">
         <v>896</v>
       </c>
-      <c r="S28" s="45" t="s">
-        <v>897</v>
-      </c>
       <c r="T28" s="45" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="U28" s="45" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="V28" s="45" t="s">
         <v>781</v>
       </c>
       <c r="W28" s="45" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="X28" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y28" s="45" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="Z28" s="47">
         <v>0</v>
@@ -15063,19 +15063,19 @@
         <v>412</v>
       </c>
       <c r="N29" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P29" s="45" t="s">
         <v>787</v>
       </c>
       <c r="R29" s="45" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="T29" s="45" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="V29" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X29" s="45" t="s">
         <v>783</v>
@@ -15110,7 +15110,7 @@
         <v>409</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E30" s="45" t="s">
         <v>410</v>
@@ -15140,7 +15140,7 @@
         <v>423</v>
       </c>
       <c r="N30" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P30" s="45" t="s">
         <v>787</v>
@@ -15149,13 +15149,13 @@
         <v>788</v>
       </c>
       <c r="T30" s="45" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="V30" s="45" t="s">
         <v>781</v>
       </c>
       <c r="W30" s="45" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="X30" s="45" t="s">
         <v>783</v>
@@ -15190,7 +15190,7 @@
         <v>409</v>
       </c>
       <c r="D31" s="46" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E31" s="45" t="s">
         <v>435</v>
@@ -15223,7 +15223,7 @@
         <v>773</v>
       </c>
       <c r="P31" s="45" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="R31" s="45" t="s">
         <v>788</v>
@@ -15232,7 +15232,7 @@
         <v>779</v>
       </c>
       <c r="V31" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X31" s="45" t="s">
         <v>783</v>
@@ -15294,19 +15294,19 @@
         <v>726</v>
       </c>
       <c r="M32" s="45" t="s">
+        <v>900</v>
+      </c>
+      <c r="N32" s="45" t="s">
+        <v>816</v>
+      </c>
+      <c r="O32" s="45" t="s">
         <v>901</v>
-      </c>
-      <c r="N32" s="45" t="s">
-        <v>817</v>
-      </c>
-      <c r="O32" s="45" t="s">
-        <v>902</v>
       </c>
       <c r="P32" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q32" s="45" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="R32" s="45" t="s">
         <v>788</v>
@@ -15315,16 +15315,16 @@
         <v>779</v>
       </c>
       <c r="U32" s="45" t="s">
+        <v>903</v>
+      </c>
+      <c r="V32" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="X32" s="45" t="s">
+        <v>870</v>
+      </c>
+      <c r="Y32" s="45" t="s">
         <v>904</v>
-      </c>
-      <c r="V32" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="X32" s="45" t="s">
-        <v>871</v>
-      </c>
-      <c r="Y32" s="45" t="s">
-        <v>905</v>
       </c>
       <c r="Z32" s="47">
         <v>3</v>
@@ -15356,7 +15356,7 @@
         <v>440</v>
       </c>
       <c r="D33" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E33" s="45" t="s">
         <v>453</v>
@@ -15383,19 +15383,19 @@
         <v>726</v>
       </c>
       <c r="M33" s="45" t="s">
+        <v>905</v>
+      </c>
+      <c r="N33" s="45" t="s">
+        <v>816</v>
+      </c>
+      <c r="O33" s="45" t="s">
         <v>906</v>
       </c>
-      <c r="N33" s="45" t="s">
-        <v>817</v>
-      </c>
-      <c r="O33" s="45" t="s">
+      <c r="P33" s="45" t="s">
+        <v>827</v>
+      </c>
+      <c r="Q33" s="45" t="s">
         <v>907</v>
-      </c>
-      <c r="P33" s="45" t="s">
-        <v>828</v>
-      </c>
-      <c r="Q33" s="45" t="s">
-        <v>908</v>
       </c>
       <c r="R33" s="45" t="s">
         <v>788</v>
@@ -15404,10 +15404,10 @@
         <v>779</v>
       </c>
       <c r="U33" s="45" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="V33" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X33" s="45" t="s">
         <v>783</v>
@@ -15469,37 +15469,37 @@
         <v>727</v>
       </c>
       <c r="M34" s="45" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="N34" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O34" s="45" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="P34" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q34" s="45" t="s">
+        <v>911</v>
+      </c>
+      <c r="R34" s="45" t="s">
+        <v>829</v>
+      </c>
+      <c r="S34" s="45" t="s">
         <v>912</v>
-      </c>
-      <c r="R34" s="45" t="s">
-        <v>830</v>
-      </c>
-      <c r="S34" s="45" t="s">
-        <v>913</v>
       </c>
       <c r="T34" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U34" s="45" t="s">
+        <v>913</v>
+      </c>
+      <c r="V34" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W34" s="45" t="s">
         <v>914</v>
-      </c>
-      <c r="V34" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W34" s="45" t="s">
-        <v>915</v>
       </c>
       <c r="X34" s="45" t="s">
         <v>783</v>
@@ -15534,7 +15534,7 @@
         <v>466</v>
       </c>
       <c r="D35" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E35" s="45" t="s">
         <v>467</v>
@@ -15561,43 +15561,43 @@
         <v>727</v>
       </c>
       <c r="M35" s="45" t="s">
+        <v>915</v>
+      </c>
+      <c r="N35" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O35" s="45" t="s">
         <v>916</v>
-      </c>
-      <c r="N35" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O35" s="45" t="s">
-        <v>917</v>
       </c>
       <c r="P35" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q35" s="45" t="s">
+        <v>917</v>
+      </c>
+      <c r="R35" s="45" t="s">
+        <v>829</v>
+      </c>
+      <c r="S35" s="45" t="s">
         <v>918</v>
-      </c>
-      <c r="R35" s="45" t="s">
-        <v>830</v>
-      </c>
-      <c r="S35" s="45" t="s">
-        <v>919</v>
       </c>
       <c r="T35" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U35" s="45" t="s">
+        <v>919</v>
+      </c>
+      <c r="V35" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W35" s="45" t="s">
         <v>920</v>
-      </c>
-      <c r="V35" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W35" s="45" t="s">
-        <v>921</v>
       </c>
       <c r="X35" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y35" s="45" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="Z35" s="47">
         <v>0</v>
@@ -15662,28 +15662,28 @@
         <v>785</v>
       </c>
       <c r="O36" s="45" t="s">
+        <v>922</v>
+      </c>
+      <c r="P36" s="45" t="s">
+        <v>827</v>
+      </c>
+      <c r="Q36" s="45" t="s">
         <v>923</v>
       </c>
-      <c r="P36" s="45" t="s">
-        <v>828</v>
-      </c>
-      <c r="Q36" s="45" t="s">
-        <v>924</v>
-      </c>
       <c r="R36" s="45" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="T36" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U36" s="45" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="V36" s="45" t="s">
         <v>789</v>
       </c>
       <c r="W36" s="45" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="X36" s="45" t="s">
         <v>783</v>
@@ -15718,7 +15718,7 @@
         <v>481</v>
       </c>
       <c r="D37" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E37" s="45" t="s">
         <v>490</v>
@@ -15760,10 +15760,10 @@
         <v>779</v>
       </c>
       <c r="U37" s="45" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="V37" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X37" s="45" t="s">
         <v>783</v>
@@ -15825,13 +15825,13 @@
         <v>729</v>
       </c>
       <c r="M38" s="45" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="N38" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O38" s="45" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="P38" s="45" t="s">
         <v>787</v>
@@ -15840,10 +15840,10 @@
         <v>788</v>
       </c>
       <c r="T38" s="45" t="s">
+        <v>793</v>
+      </c>
+      <c r="V38" s="45" t="s">
         <v>794</v>
-      </c>
-      <c r="V38" s="45" t="s">
-        <v>795</v>
       </c>
       <c r="X38" s="45" t="s">
         <v>783</v>
@@ -15911,28 +15911,28 @@
         <v>773</v>
       </c>
       <c r="O39" s="45" t="s">
+        <v>929</v>
+      </c>
+      <c r="P39" s="45" t="s">
+        <v>827</v>
+      </c>
+      <c r="Q39" s="45" t="s">
         <v>930</v>
       </c>
-      <c r="P39" s="45" t="s">
-        <v>828</v>
-      </c>
-      <c r="Q39" s="45" t="s">
+      <c r="R39" s="45" t="s">
+        <v>829</v>
+      </c>
+      <c r="T39" s="45" t="s">
+        <v>793</v>
+      </c>
+      <c r="U39" s="45" t="s">
         <v>931</v>
       </c>
-      <c r="R39" s="45" t="s">
-        <v>830</v>
-      </c>
-      <c r="T39" s="45" t="s">
+      <c r="V39" s="45" t="s">
         <v>794</v>
       </c>
-      <c r="U39" s="45" t="s">
+      <c r="W39" s="45" t="s">
         <v>932</v>
-      </c>
-      <c r="V39" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W39" s="45" t="s">
-        <v>933</v>
       </c>
       <c r="X39" s="45" t="s">
         <v>783</v>
@@ -15994,31 +15994,31 @@
         <v>731</v>
       </c>
       <c r="M40" s="45" t="s">
+        <v>933</v>
+      </c>
+      <c r="N40" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="P40" s="45" t="s">
         <v>934</v>
-      </c>
-      <c r="N40" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="P40" s="45" t="s">
-        <v>935</v>
       </c>
       <c r="R40" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S40" s="45" t="s">
+        <v>935</v>
+      </c>
+      <c r="T40" s="45" t="s">
+        <v>793</v>
+      </c>
+      <c r="U40" s="45" t="s">
         <v>936</v>
       </c>
-      <c r="T40" s="45" t="s">
+      <c r="V40" s="45" t="s">
         <v>794</v>
       </c>
-      <c r="U40" s="45" t="s">
+      <c r="W40" s="45" t="s">
         <v>937</v>
-      </c>
-      <c r="V40" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W40" s="45" t="s">
-        <v>938</v>
       </c>
       <c r="X40" s="45" t="s">
         <v>783</v>
@@ -16053,7 +16053,7 @@
         <v>526</v>
       </c>
       <c r="D41" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E41" s="45" t="s">
         <v>527</v>
@@ -16080,43 +16080,43 @@
         <v>731</v>
       </c>
       <c r="M41" s="45" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="N41" s="45" t="s">
         <v>785</v>
       </c>
       <c r="O41" s="45" t="s">
+        <v>939</v>
+      </c>
+      <c r="P41" s="45" t="s">
+        <v>879</v>
+      </c>
+      <c r="Q41" s="45" t="s">
         <v>940</v>
-      </c>
-      <c r="P41" s="45" t="s">
-        <v>880</v>
-      </c>
-      <c r="Q41" s="45" t="s">
-        <v>941</v>
       </c>
       <c r="R41" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S41" s="45" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="T41" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U41" s="45" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="V41" s="45" t="s">
         <v>789</v>
       </c>
       <c r="W41" s="45" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="X41" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y41" s="45" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="Z41" s="47">
         <v>2</v>
@@ -16142,7 +16142,7 @@
         <v>38</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="C42" s="46" t="s">
         <v>540</v>
@@ -16172,28 +16172,28 @@
         <v>148</v>
       </c>
       <c r="L42" s="1" t="s">
+        <v>945</v>
+      </c>
+      <c r="M42" s="45" t="s">
         <v>946</v>
       </c>
-      <c r="M42" s="45" t="s">
-        <v>947</v>
-      </c>
       <c r="N42" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P42" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q42" s="45" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="R42" s="45" t="s">
         <v>788</v>
       </c>
       <c r="T42" s="45" t="s">
+        <v>793</v>
+      </c>
+      <c r="V42" s="45" t="s">
         <v>794</v>
-      </c>
-      <c r="V42" s="45" t="s">
-        <v>795</v>
       </c>
       <c r="X42" s="45" t="s">
         <v>783</v>
@@ -16258,19 +16258,19 @@
         <v>234</v>
       </c>
       <c r="N43" s="45" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="P43" s="45" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="R43" s="45" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="T43" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U43" s="45" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="V43" s="45" t="s">
         <v>781</v>
@@ -16335,16 +16335,16 @@
         <v>734</v>
       </c>
       <c r="M44" s="45" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="N44" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P44" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q44" s="45" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="R44" s="45" t="s">
         <v>788</v>
@@ -16353,7 +16353,7 @@
         <v>779</v>
       </c>
       <c r="V44" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X44" s="45" t="s">
         <v>783</v>
@@ -16388,7 +16388,7 @@
         <v>552</v>
       </c>
       <c r="D45" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E45" s="45" t="s">
         <v>556</v>
@@ -16415,13 +16415,13 @@
         <v>734</v>
       </c>
       <c r="M45" s="45" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="N45" s="45" t="s">
         <v>785</v>
       </c>
       <c r="O45" s="45" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="P45" s="45" t="s">
         <v>775</v>
@@ -16495,37 +16495,37 @@
         <v>736</v>
       </c>
       <c r="M46" s="45" t="s">
+        <v>953</v>
+      </c>
+      <c r="N46" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O46" s="45" t="s">
         <v>954</v>
-      </c>
-      <c r="N46" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O46" s="45" t="s">
-        <v>955</v>
       </c>
       <c r="P46" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q46" s="45" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="R46" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S46" s="45" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="T46" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U46" s="45" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="V46" s="45" t="s">
         <v>789</v>
       </c>
       <c r="W46" s="45" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="X46" s="45" t="s">
         <v>783</v>
@@ -16554,7 +16554,7 @@
         <v>38</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="C47" s="46" t="s">
         <v>572</v>
@@ -16584,46 +16584,46 @@
         <v>103</v>
       </c>
       <c r="L47" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="M47" s="45" t="s">
         <v>960</v>
-      </c>
-      <c r="M47" s="45" t="s">
-        <v>961</v>
       </c>
       <c r="N47" s="45" t="s">
         <v>785</v>
       </c>
       <c r="O47" s="45" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="P47" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q47" s="45" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="R47" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S47" s="45" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="T47" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U47" s="45" t="s">
+        <v>964</v>
+      </c>
+      <c r="V47" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W47" s="45" t="s">
         <v>965</v>
-      </c>
-      <c r="V47" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W47" s="45" t="s">
-        <v>966</v>
       </c>
       <c r="X47" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y47" s="45" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="Z47" s="47">
         <v>2</v>
@@ -16670,7 +16670,7 @@
         <v>69</v>
       </c>
       <c r="I48" s="45" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="J48" t="s">
         <v>709</v>
@@ -16682,7 +16682,7 @@
         <v>738</v>
       </c>
       <c r="M48" s="45" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="N48" s="45" t="s">
         <v>785</v>
@@ -16697,7 +16697,7 @@
         <v>779</v>
       </c>
       <c r="V48" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X48" s="45" t="s">
         <v>783</v>
@@ -16732,7 +16732,7 @@
         <v>586</v>
       </c>
       <c r="D49" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E49" s="45" t="s">
         <v>587</v>
@@ -16759,19 +16759,19 @@
         <v>738</v>
       </c>
       <c r="M49" s="45" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="N49" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O49" s="45" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="P49" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q49" s="45" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="R49" s="45" t="s">
         <v>788</v>
@@ -16780,10 +16780,10 @@
         <v>779</v>
       </c>
       <c r="U49" s="45" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="V49" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X49" s="45" t="s">
         <v>783</v>
@@ -16845,43 +16845,43 @@
         <v>739</v>
       </c>
       <c r="M50" s="45" t="s">
+        <v>973</v>
+      </c>
+      <c r="N50" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O50" s="45" t="s">
         <v>974</v>
-      </c>
-      <c r="N50" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O50" s="45" t="s">
-        <v>975</v>
       </c>
       <c r="P50" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q50" s="45" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="R50" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S50" s="45" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="T50" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U50" s="45" t="s">
+        <v>977</v>
+      </c>
+      <c r="V50" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W50" s="45" t="s">
         <v>978</v>
-      </c>
-      <c r="V50" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W50" s="45" t="s">
-        <v>979</v>
       </c>
       <c r="X50" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y50" s="45" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="Z50" s="47">
         <v>0</v>
@@ -16940,25 +16940,25 @@
         <v>740</v>
       </c>
       <c r="M51" s="45" t="s">
+        <v>980</v>
+      </c>
+      <c r="N51" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="P51" s="45" t="s">
+        <v>879</v>
+      </c>
+      <c r="Q51" s="45" t="s">
         <v>981</v>
-      </c>
-      <c r="N51" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="P51" s="45" t="s">
-        <v>880</v>
-      </c>
-      <c r="Q51" s="45" t="s">
-        <v>982</v>
       </c>
       <c r="R51" s="45" t="s">
         <v>788</v>
       </c>
       <c r="T51" s="45" t="s">
+        <v>793</v>
+      </c>
+      <c r="V51" s="45" t="s">
         <v>794</v>
-      </c>
-      <c r="V51" s="45" t="s">
-        <v>795</v>
       </c>
       <c r="X51" s="45" t="s">
         <v>783</v>
@@ -17020,37 +17020,37 @@
         <v>741</v>
       </c>
       <c r="M52" s="45" t="s">
+        <v>982</v>
+      </c>
+      <c r="N52" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O52" s="45" t="s">
         <v>983</v>
-      </c>
-      <c r="N52" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O52" s="45" t="s">
-        <v>984</v>
       </c>
       <c r="P52" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q52" s="45" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="R52" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S52" s="45" t="s">
+        <v>985</v>
+      </c>
+      <c r="T52" s="45" t="s">
+        <v>811</v>
+      </c>
+      <c r="U52" s="45" t="s">
         <v>986</v>
       </c>
-      <c r="T52" s="45" t="s">
-        <v>812</v>
-      </c>
-      <c r="U52" s="45" t="s">
+      <c r="V52" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W52" s="45" t="s">
         <v>987</v>
-      </c>
-      <c r="V52" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W52" s="45" t="s">
-        <v>988</v>
       </c>
       <c r="X52" s="45" t="s">
         <v>783</v>
@@ -17115,43 +17115,43 @@
         <v>742</v>
       </c>
       <c r="M53" s="45" t="s">
+        <v>988</v>
+      </c>
+      <c r="N53" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O53" s="45" t="s">
         <v>989</v>
-      </c>
-      <c r="N53" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O53" s="45" t="s">
-        <v>990</v>
       </c>
       <c r="P53" s="45" t="s">
         <v>787</v>
       </c>
       <c r="Q53" s="45" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="R53" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S53" s="45" t="s">
+        <v>991</v>
+      </c>
+      <c r="T53" s="45" t="s">
+        <v>881</v>
+      </c>
+      <c r="U53" s="45" t="s">
         <v>992</v>
       </c>
-      <c r="T53" s="45" t="s">
-        <v>882</v>
-      </c>
-      <c r="U53" s="45" t="s">
+      <c r="V53" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W53" s="45" t="s">
         <v>993</v>
-      </c>
-      <c r="V53" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W53" s="45" t="s">
-        <v>994</v>
       </c>
       <c r="X53" s="45" t="s">
         <v>783</v>
       </c>
       <c r="Y53" s="45" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="Z53" s="47">
         <v>0</v>
@@ -17183,7 +17183,7 @@
         <v>646</v>
       </c>
       <c r="D54" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E54" s="45" t="s">
         <v>652</v>
@@ -17210,31 +17210,31 @@
         <v>743</v>
       </c>
       <c r="M54" s="45" t="s">
+        <v>995</v>
+      </c>
+      <c r="N54" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="P54" s="45" t="s">
+        <v>879</v>
+      </c>
+      <c r="Q54" s="45" t="s">
         <v>996</v>
-      </c>
-      <c r="N54" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="P54" s="45" t="s">
-        <v>880</v>
-      </c>
-      <c r="Q54" s="45" t="s">
-        <v>997</v>
       </c>
       <c r="R54" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S54" s="45" t="s">
+        <v>997</v>
+      </c>
+      <c r="T54" s="45" t="s">
+        <v>811</v>
+      </c>
+      <c r="U54" s="45" t="s">
         <v>998</v>
       </c>
-      <c r="T54" s="45" t="s">
-        <v>812</v>
-      </c>
-      <c r="U54" s="45" t="s">
-        <v>999</v>
-      </c>
       <c r="V54" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X54" s="45" t="s">
         <v>783</v>
@@ -17269,7 +17269,7 @@
         <v>646</v>
       </c>
       <c r="D55" s="46" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E55" s="45" t="s">
         <v>657</v>
@@ -17296,7 +17296,7 @@
         <v>743</v>
       </c>
       <c r="M55" s="45" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="N55" s="45" t="s">
         <v>785</v>
@@ -17308,10 +17308,10 @@
         <v>788</v>
       </c>
       <c r="T55" s="45" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="V55" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X55" s="45" t="s">
         <v>783</v>
@@ -17373,10 +17373,10 @@
         <v>743</v>
       </c>
       <c r="M56" s="45" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="N56" s="45" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="P56" s="45" t="s">
         <v>787</v>
@@ -17385,13 +17385,13 @@
         <v>788</v>
       </c>
       <c r="S56" s="45" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="T56" s="45" t="s">
         <v>779</v>
       </c>
       <c r="V56" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X56" s="45" t="s">
         <v>783</v>
@@ -17453,7 +17453,7 @@
         <v>744</v>
       </c>
       <c r="M57" s="45" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="N57" s="45" t="s">
         <v>773</v>
@@ -17465,7 +17465,7 @@
         <v>777</v>
       </c>
       <c r="T57" s="45" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="V57" s="45" t="s">
         <v>789</v>
@@ -17530,34 +17530,34 @@
         <v>745</v>
       </c>
       <c r="M58" s="45" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="N58" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O58" s="45" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="P58" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q58" s="45" t="s">
+        <v>1005</v>
+      </c>
+      <c r="R58" s="45" t="s">
+        <v>895</v>
+      </c>
+      <c r="S58" s="45" t="s">
         <v>1006</v>
-      </c>
-      <c r="R58" s="45" t="s">
-        <v>896</v>
-      </c>
-      <c r="S58" s="45" t="s">
-        <v>1007</v>
       </c>
       <c r="T58" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U58" s="45" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="V58" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X58" s="45" t="s">
         <v>783</v>
@@ -17592,7 +17592,7 @@
         <v>665</v>
       </c>
       <c r="D59" s="46" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E59" s="45" t="s">
         <v>40</v>
@@ -17619,34 +17619,34 @@
         <v>745</v>
       </c>
       <c r="M59" s="45" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="N59" s="45" t="s">
         <v>773</v>
       </c>
       <c r="O59" s="45" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="P59" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q59" s="45" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="R59" s="45" t="s">
         <v>788</v>
       </c>
       <c r="S59" s="45" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="T59" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U59" s="45" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="V59" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X59" s="45" t="s">
         <v>783</v>
@@ -17681,7 +17681,7 @@
         <v>665</v>
       </c>
       <c r="D60" s="46" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="E60" s="45" t="s">
         <v>40</v>
@@ -17708,34 +17708,34 @@
         <v>745</v>
       </c>
       <c r="M60" s="45" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="N60" s="45" t="s">
         <v>785</v>
       </c>
       <c r="O60" s="45" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="P60" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q60" s="45" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="R60" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S60" s="45" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="T60" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U60" s="45" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="V60" s="45" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="X60" s="45" t="s">
         <v>783</v>
@@ -17797,37 +17797,37 @@
         <v>746</v>
       </c>
       <c r="M61" s="45" t="s">
+        <v>1017</v>
+      </c>
+      <c r="N61" s="45" t="s">
+        <v>804</v>
+      </c>
+      <c r="O61" s="45" t="s">
         <v>1018</v>
-      </c>
-      <c r="N61" s="45" t="s">
-        <v>805</v>
-      </c>
-      <c r="O61" s="45" t="s">
-        <v>1019</v>
       </c>
       <c r="P61" s="45" t="s">
         <v>775</v>
       </c>
       <c r="Q61" s="45" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="R61" s="45" t="s">
         <v>777</v>
       </c>
       <c r="S61" s="45" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="T61" s="45" t="s">
         <v>779</v>
       </c>
       <c r="U61" s="45" t="s">
+        <v>1021</v>
+      </c>
+      <c r="V61" s="45" t="s">
+        <v>794</v>
+      </c>
+      <c r="W61" s="45" t="s">
         <v>1022</v>
-      </c>
-      <c r="V61" s="45" t="s">
-        <v>795</v>
-      </c>
-      <c r="W61" s="45" t="s">
-        <v>1023</v>
       </c>
       <c r="X61" s="45" t="s">
         <v>783</v>
@@ -17865,12 +17865,12 @@
       <c r="E62" s="48"/>
       <c r="F62" s="48"/>
       <c r="G62" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="H62" s="48"/>
       <c r="I62" s="48"/>
       <c r="J62" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="K62" s="48"/>
       <c r="L62" s="20" t="s">
@@ -17910,12 +17910,12 @@
       <c r="E63" s="48"/>
       <c r="F63" s="48"/>
       <c r="G63" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="H63" s="48"/>
       <c r="I63" s="48"/>
       <c r="J63" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="K63" s="48"/>
       <c r="L63" s="9" t="s">
@@ -17931,7 +17931,7 @@
       <c r="T63" s="48"/>
       <c r="U63" s="48"/>
       <c r="V63" s="48" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="W63" s="48"/>
       <c r="X63" s="48" t="s">
@@ -17963,12 +17963,12 @@
       <c r="E64" s="48"/>
       <c r="F64" s="48"/>
       <c r="G64" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="H64" s="48"/>
       <c r="I64" s="48"/>
       <c r="J64" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="K64" s="48"/>
       <c r="L64" s="9" t="s">
@@ -17999,7 +17999,7 @@
         <v>548</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="C65" s="49" t="s">
         <v>703</v>
@@ -18008,16 +18008,16 @@
       <c r="E65" s="48"/>
       <c r="F65" s="48"/>
       <c r="G65" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="H65" s="48"/>
       <c r="I65" s="48"/>
       <c r="J65" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="K65" s="48"/>
       <c r="L65" s="9" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="M65" s="48"/>
       <c r="N65" s="48"/>
@@ -18053,12 +18053,12 @@
       <c r="E66" s="48"/>
       <c r="F66" s="48"/>
       <c r="G66" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="H66" s="48"/>
       <c r="I66" s="48"/>
       <c r="J66" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="K66" s="48"/>
       <c r="L66" s="25" t="s">
@@ -18089,25 +18089,25 @@
         <v>548</v>
       </c>
       <c r="B67" s="51" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C67" s="49" t="s">
         <v>1026</v>
-      </c>
-      <c r="C67" s="49" t="s">
-        <v>1027</v>
       </c>
       <c r="D67" s="49"/>
       <c r="E67" s="48"/>
       <c r="F67" s="48"/>
       <c r="G67" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="H67" s="48"/>
       <c r="I67" s="48"/>
       <c r="J67" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="K67" s="48"/>
       <c r="L67" s="51" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="M67" s="48"/>
       <c r="N67" s="48"/>

</xml_diff>